<commit_message>
Update notebook with base-100 index plots and save to plots/ folder
- Rewrote cumulative performance plots to use base 100 (standard finance convention)
- Added distinctive styling: custom colors, filled areas, end-value annotations, group watermark
- Generated and saved individual PNGs for VW and MV portfolios in plots/
- Expanded Part_I_Explanation.md to cover every code line

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Part_1.xlsx
+++ b/Part_1.xlsx
@@ -8,25 +8,32 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TOTO2\PycharmProjects\SAAM-Project-2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{40AF2E89-7B48-4755-9394-452DCB8AE7E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97A6F049-983B-4720-9513-E14CFA60DAC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="12">
-  <si>
-    <t>Characteristics of portfolio (Please provide real numbers instead of percentages. For example, use 0.02 instead of 2%.)</t>
-  </si>
-  <si>
-    <t>Monthly Portfolio returns (Please provide real numbers instead of percentages. For example, use 0.02 instead of 2%.)</t>
-  </si>
   <si>
     <t>Value-weighted portfolio</t>
   </si>
@@ -56,6 +63,12 @@
   </si>
   <si>
     <t>(insert your plot here)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Characteristics of portfolio </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monthly Portfolio returns </t>
   </si>
 </sst>
 </file>
@@ -296,22 +309,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>9525</xdr:rowOff>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>9524</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>135373</xdr:rowOff>
+      <xdr:colOff>781051</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>158947</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1">
+        <xdr:cNvPr id="9" name="Picture 8">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6A060F4F-8F49-4DE6-0EE8-60CD74740111}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{94C2AF35-383E-12D7-CC0B-59BB1563D989}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -320,15 +333,21 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="1838325"/>
-          <a:ext cx="7629524" cy="3126223"/>
+          <a:off x="1" y="2181225"/>
+          <a:ext cx="8401050" cy="3807022"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -340,22 +359,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>38101</xdr:rowOff>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>128587</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>2806071</xdr:colOff>
-      <xdr:row>40</xdr:row>
-      <xdr:rowOff>142876</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>819151</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>152399</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 3">
+        <xdr:cNvPr id="11" name="Picture 10">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E65C20B4-691F-5AAF-211F-41FA2FCC1959}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{864F5436-C96F-2689-FE06-E45353D02763}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -377,8 +396,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="5067301"/>
-          <a:ext cx="7578096" cy="3105150"/>
+          <a:off x="1" y="6157912"/>
+          <a:ext cx="8439150" cy="3824287"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -720,12 +739,12 @@
   <sheetData>
     <row r="1" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="B1" s="13"/>
       <c r="C1" s="14"/>
       <c r="E1" s="12" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="F1" s="13"/>
       <c r="G1" s="14"/>
@@ -733,22 +752,22 @@
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="15"/>
       <c r="B2" s="16" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E2" s="8"/>
       <c r="F2" s="6" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B3">
         <v>0.1141873277142665</v>
@@ -768,7 +787,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B4">
         <v>0.14206157228384081</v>
@@ -788,7 +807,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B5">
         <v>0.1092552439921162</v>
@@ -808,7 +827,7 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B6">
         <v>0.7936685828921507</v>
@@ -828,7 +847,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B7">
         <v>-0.13183697197203301</v>
@@ -848,7 +867,7 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B8">
         <v>0.12913082323572189</v>
@@ -868,11 +887,11 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B9" s="18"/>
       <c r="C9" s="19" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E9" s="9">
         <v>41851</v>

</xml_diff>